<commit_message>
changed implementation from deterministic python sorting algo to agentic
</commit_message>
<xml_diff>
--- a/test_rooms.xlsx
+++ b/test_rooms.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,13 +481,43 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>CR-104</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>classroom</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>LAB-201</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B6" t="n">
         <v>30</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LAB-202</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t>lab</t>
         </is>

</xml_diff>